<commit_message>
Markdown knowledge base and updated code base
</commit_message>
<xml_diff>
--- a/source_docs/Ithaka-Portico-KnowledgeBase.xlsx
+++ b/source_docs/Ithaka-Portico-KnowledgeBase.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://innodata-my.sharepoint.com/personal/vff_innodata_com/Documents/Shared with Everyone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A90B196-F6B6-4511-B917-773D6A39D8E7}"/>
+  <xr:revisionPtr revIDLastSave="450" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5890746-5E04-45E4-BA60-06D5E034FCD7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="WorkBench-Errors-Resolution" sheetId="1" r:id="rId1"/>
+    <sheet name="00_DOMAINS_AND_METADATA" sheetId="2" r:id="rId1"/>
+    <sheet name="WorkBench-Errors-Resolution" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="118">
   <si>
     <t>Developer</t>
   </si>
@@ -56,9 +57,6 @@
     <t>Knowledge Source</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
     <t>Jira/Email detail</t>
   </si>
   <si>
@@ -69,9 +67,6 @@
   </si>
   <si>
     <t>MICROBIO-BL-SETUP-24610</t>
-  </si>
-  <si>
-    <t>C550</t>
   </si>
   <si>
     <t>TOOL032 - Bad data: Value of 'xml:lang' attribute of element ref not equal to a RFC 3066 value (as defined by ISO 639-1 | ISO 639-2 | ISO 639-3). 
@@ -161,6 +156,9 @@
 - Final Resolution: Script Fix</t>
   </si>
   <si>
+    <t>C550</t>
+  </si>
+  <si>
     <t>TOOL001 - QCA774, Bad data: Value of 'country' attribute of element country not equal to codes defined by ISO in ISO 3166 and listed at: http://www.iso.org/iso/country_codes/iso_3166_code_lists.htm. These codes are subject to change, so if this error is raised, be sure to check the ISO web site to see if this is a genuine error, or if thePortico Schematron file must be updated to include a new value.:::/article[1]/front[1]/article-meta[1]/aff[1]/country[1]</t>
   </si>
   <si>
@@ -411,16 +409,127 @@
     <t>- Month must be present in [ pub-date ] when Year and Day are given.
 - Resolution: Script logiv FIXED template "pub-date"</t>
   </si>
+  <si>
+    <t>PORTLAND JATS E-Journals - BL-SETUP-24894</t>
+  </si>
+  <si>
+    <t>C512</t>
+  </si>
+  <si>
+    <t>C512 : SU 13 (Category: Processing) Step : PorticoWorkflow_4_3_ResolveFileReferences
+No file found for the token 'ETLS-2025-3021.pdf' referenced in the generated(target) lead MD file etls/237353/etls-2025-3021-xml/conprep_generated/tms3qc7v3nn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Dropping Reference of PDF File for Full-Text Content.
+- Publisher confirmed that PDF file not available on Publisher's website
+- Resolution: we are dropping the reference to the PDF file from the element 'self-uri'.
+</t>
+  </si>
+  <si>
+    <t>NAPC JATS E-Journals</t>
+  </si>
+  <si>
+    <t>C550 (Category: Tool) Step : PorticoWorkflow_4_3_ReplaceFileReferences
+Automated QC detected errors in the generated(target) lead MD file ajas/ajas_5_1502/ajas-xml/conprep_generated/tms3xzm0666
+Messages Content:
+TOOL001 - QCA753, Programming exception: Element abstract should have a title and does not.:::/article[1]/front[1]/article-meta[1]/abstract[1]
+TOOL001 - QCA753, Programming exception: Element kwd-group should have a title and does not.:::/article[1]/front[1]/article-meta[1]/kwd-group[1]</t>
+  </si>
+  <si>
+    <t>- Publisher has not provided title element in the abstract and kwd-group
+- Resolution: We are genrating the title element in the output through "insert-titles-jats.xsl" script.</t>
+  </si>
+  <si>
+    <t>C550 : SU 61 (Category: Tool) Step : PorticoWorkflow_4_3_ReplaceFileReferences
+Automated QC detected errors in the generated(target) lead MD file bio/237596/bio-2026-203-xml/conprep_generated/tms3q1c6gm8</t>
+  </si>
+  <si>
+    <t>- Element graphic should have a position attribute equal to 'anchor'.
+- Resolution: We updated the transformation script to change the position attribute equal to 'anchor'.</t>
+  </si>
+  <si>
+    <t>WSPC ATY E-Journals-SETUP-25056</t>
+  </si>
+  <si>
+    <t>C500 : SU 17 (Category: Processing) Step : PorticoWorkflow_4_3_TransformFiles
+Failed to transform the supplied file ac.33.issue-02_20260512194254.zip/s1005386726000180/s1005386726000180.xml</t>
+  </si>
+  <si>
+    <t>- Unhandled Value of Attribute '@rid' and '@id'
+- Resolution: We updated the transformation script to handled the ID and RID issues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- A sequence of more than one item is not allowed as the first argument of fn:normalize-space()
+- Resolution: We updated the transformation script to handled these type issues.
+</t>
+  </si>
+  <si>
+    <t>C464 (Category: Processing) Step : PorticoWorkflow_4_3_TransformFiles
+Generated file ajas/ajas_5_1502/ajas-xml/conprep_generated/tms3xzp1nbh well-formed but not valid.
+Messages Content:
+TOOL014 - The file is well-formed but not valid for the format: PTC_JATS_Archiving_MML2_DTD_1.3
+SAXParseException. Attribute "content-type" must be declared for element type "ext-link". Line = 14, Column = 200.SAXParseException. The content of element type "article-meta" must match "(article-id*,(article-version|article-version-alternatives)?,article-categories?,title-group?,(contrib-group|aff|aff-alternatives|x)*,author-notes?,(pub-date*|pub-date-not-available?),volume*,volume-id*,volume-series?,issue*,issue-id*,issue-title*,issue-title-group*,issue-sponsor*,issue-part?,volume-issue-group*,isbn*,supplement?,(((fpage,lpage?)?,page-range?)|elocation-id)?,(email|ext-link|uri|product|supplementary-material)*,history?,pub-history?,permissions?,self-uri*,(related-article|related-object)*,abstract*,trans-abstract*,kwd-group*,funding-group*,support-group*,conference*,counts?,custom-meta-group?)". Line = 14, Column = 2,304.</t>
+  </si>
+  <si>
+    <t>- Attribute @content-type is not valid as per the PTC output format.
+- Resolution: We need to updating the transform script and resolved this issue.</t>
+  </si>
+  <si>
+    <t>C448 (Category: Configuration) Step : PorticoWorkflow_4_3_CheckForCompleteness
+Orphan File /pcontent/ongoing/journal_content/INGEST_MASTER/NAPC/Fetched/SELF/NEW/nap_portico_complete/ajas_5_1_2013.zip/_manifest.txt: not fully unit identified.
+Messages Content:
+Check file naming and Profile rules</t>
+  </si>
+  <si>
+    <t>- Publisher porvided the extra files in the ZIP.
+- Resolution: If we are not able to group any file in the any CU and publisher not provided reference of provided file we have checked this file and exculde such type file through FER rule.</t>
+  </si>
+  <si>
+    <t>MRE JATS E-Journals-SETUP-25050</t>
+  </si>
+  <si>
+    <t>Orphan File /pcontent/ongoing/journal_content/INGEST_MASTER/MRE/Fetched/JATS/NEW/SV/SV_18_2_2022.zip/SV_18_2_2022/SV2021050701/SV2021050701_Immediate_Effect_Supplement_1.docx: not fully unit identified.</t>
+  </si>
+  <si>
+    <t>- Supplementary files are not getting to identified by the current rule 'InterpretPackagingRuleSet'
+- Resolution: We updated the associated rule and now files are correct identified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orphan File /pcontent/ongoing/journal_content/INGEST_MASTER/MRE/Fetched/JATS/NEW/EJGO/EJGO_43_3_2022.zip/EJGO_43_3_2022/EJGO22012001/video1.png: not fully unit identified.
+</t>
+  </si>
+  <si>
+    <t>- Image files are not getting to identified by the current rule 'InterpretPackagingRuleSet'
+- Resolution: We updated the associated rule and now files are correct identified</t>
+  </si>
+  <si>
+    <t>C464 : SU 85 (Category: Processing) Step : PorticoWorkflow_4_3_TransformFiles
+Generated file EMERALD E-Books/978-1-59311-357-5/xml/conprep_generated/tms2gvmxdb1 well-formed but not valid.</t>
+  </si>
+  <si>
+    <t>Sheet Category</t>
+  </si>
+  <si>
+    <t>Document Domain</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Technical Workbench Logs</t>
+  </si>
+  <si>
+    <t>PROJECT ERROR LOG DATABASE</t>
+  </si>
+  <si>
+    <t>Contains error codes, stream configurations, developers, and resolution steps.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-  </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +543,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -490,7 +604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -531,15 +645,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -555,17 +660,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="3"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -585,22 +694,6 @@
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom/>
-      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -767,17 +860,20 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8218E10-27D8-4199-A310-EF2F29294419}" name="Table1" displayName="Table1" ref="A1:I27" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I27" xr:uid="{C8218E10-27D8-4199-A310-EF2F29294419}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{4D214576-3A2A-4EA3-942A-5AE0C4D921C8}" name="Developer" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{40FC3A1A-F761-4C4C-A092-BFC0BB2013D7}" name="Stream Name-Setup Number" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{EFCB3567-1A5D-4AFB-8DC4-59FFC628D30D}" name="WorkBench Error Code" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7BC6EB0D-5B6A-40D8-9197-2C776DF2E3DE}" name="Error Message" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{AF06E84F-EC79-4156-A4F7-D8B35E587215}" name="Category (Transformation/Profile/Other)" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{8164D0A7-56C6-4CF7-B6C8-C446F24CC5FA}" name="Knowledge Source" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{017257B6-2629-45C5-8F8A-C4B26B3B906C}" name="Date" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8218E10-27D8-4199-A310-EF2F29294419}" name="Table1" displayName="Table1" ref="A1:H36" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H36" xr:uid="{C8218E10-27D8-4199-A310-EF2F29294419}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{4D214576-3A2A-4EA3-942A-5AE0C4D921C8}" name="Developer" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{40FC3A1A-F761-4C4C-A092-BFC0BB2013D7}" name="Stream Name-Setup Number" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{EFCB3567-1A5D-4AFB-8DC4-59FFC628D30D}" name="WorkBench Error Code" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7BC6EB0D-5B6A-40D8-9197-2C776DF2E3DE}" name="Error Message" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{AF06E84F-EC79-4156-A4F7-D8B35E587215}" name="Category (Transformation/Profile/Other)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{8164D0A7-56C6-4CF7-B6C8-C446F24CC5FA}" name="Knowledge Source" dataDxfId="2"/>
     <tableColumn id="9" xr3:uid="{9343B300-6B21-4EDE-A0BF-54FD39302602}" name="Jira/Email detail" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{5E52460C-1D9C-4EBB-9277-AFA43E689BA1}" name="Resolution Steps" dataDxfId="0"/>
   </tableColumns>
@@ -1101,18 +1197,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3775EE33-B872-4E10-90AB-177DCEAAC69A}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="65.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="40.5703125" style="2" customWidth="1"/>
     <col min="3" max="3" width="16.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="77" style="8" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" style="21" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" style="17" customWidth="1"/>
-    <col min="8" max="8" width="29.42578125" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" style="18" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" style="14" customWidth="1"/>
+    <col min="8" max="8" width="41.7109375" customWidth="1"/>
     <col min="9" max="9" width="95.28515625" customWidth="1"/>
     <col min="10" max="10" width="110.5703125" style="12" customWidth="1"/>
   </cols>
@@ -1133,636 +1266,811 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>8</v>
       </c>
       <c r="J1"/>
     </row>
     <row r="2" spans="1:10" ht="65.25" customHeight="1">
       <c r="A2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="15"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="10" t="s">
-        <v>15</v>
       </c>
       <c r="J2"/>
     </row>
     <row r="3" spans="1:10" ht="102" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="15"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="J3"/>
     </row>
     <row r="4" spans="1:10" ht="65.25" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="F4" s="15"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="18"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="10" t="s">
-        <v>22</v>
       </c>
       <c r="J4"/>
     </row>
     <row r="5" spans="1:10" ht="112.5" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="15"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="10" t="s">
-        <v>27</v>
       </c>
       <c r="J5"/>
     </row>
     <row r="6" spans="1:10" ht="141" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="16"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="11" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="19"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="11" t="s">
-        <v>32</v>
       </c>
       <c r="J6"/>
     </row>
     <row r="7" spans="1:10" ht="96.75" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="16"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="11" t="s">
         <v>33</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="11" t="s">
-        <v>34</v>
       </c>
       <c r="J7"/>
     </row>
     <row r="8" spans="1:10" ht="65.25" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="J8"/>
     </row>
     <row r="9" spans="1:10" ht="65.25" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="16"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="11" t="s">
         <v>40</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="11" t="s">
-        <v>41</v>
       </c>
       <c r="J9"/>
     </row>
     <row r="10" spans="1:10" ht="65.25" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="16"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="11" t="s">
-        <v>44</v>
       </c>
       <c r="J10"/>
     </row>
     <row r="11" spans="1:10" ht="65.25" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="E11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="16"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="11" t="s">
         <v>48</v>
-      </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="11" t="s">
-        <v>49</v>
       </c>
       <c r="J11"/>
     </row>
     <row r="12" spans="1:10" ht="65.25" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="16"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="19"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="11" t="s">
-        <v>51</v>
       </c>
       <c r="J12"/>
     </row>
     <row r="13" spans="1:10" ht="65.25" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="16"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="11" t="s">
-        <v>53</v>
       </c>
       <c r="J13"/>
     </row>
     <row r="14" spans="1:10" ht="65.25" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="16"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="11" t="s">
         <v>54</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="J14"/>
     </row>
     <row r="15" spans="1:10" ht="65.25" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="16"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="F15" s="19"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="J15"/>
     </row>
     <row r="16" spans="1:10" ht="65.25" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D16" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="11" t="s">
         <v>58</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="19"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="11" t="s">
-        <v>59</v>
       </c>
       <c r="J16"/>
     </row>
     <row r="17" spans="1:10" ht="65.25" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="11" t="s">
         <v>60</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="11" t="s">
-        <v>61</v>
       </c>
       <c r="J17"/>
     </row>
     <row r="18" spans="1:10" ht="65.25" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="16"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="J18"/>
     </row>
     <row r="19" spans="1:10" ht="65.25" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="16"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="11" t="s">
         <v>64</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="19"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="11" t="s">
-        <v>65</v>
       </c>
       <c r="J19"/>
     </row>
     <row r="20" spans="1:10" ht="65.25" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="16"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="11" t="s">
         <v>66</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="11" t="s">
-        <v>67</v>
       </c>
       <c r="J20"/>
     </row>
     <row r="21" spans="1:10" ht="65.25" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D21" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="16"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="19"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="J21"/>
     </row>
     <row r="22" spans="1:10" ht="65.25" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D22" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="16"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="19"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="J22"/>
     </row>
     <row r="23" spans="1:10" ht="65.25" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="13" t="s">
+      <c r="E23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="16"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="11" t="s">
         <v>73</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="11" t="s">
-        <v>74</v>
       </c>
       <c r="J23"/>
     </row>
     <row r="24" spans="1:10" ht="92.25" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="E24" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="G24" s="2"/>
+      <c r="H24" s="11" t="s">
         <v>79</v>
-      </c>
-      <c r="G24" s="16">
-        <v>46191</v>
-      </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="11" t="s">
-        <v>80</v>
       </c>
       <c r="J24"/>
     </row>
     <row r="25" spans="1:10" ht="65.25" customHeight="1">
       <c r="A25" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="C25" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="E25" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="F25" s="16"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="F25" s="19"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="11" t="s">
-        <v>85</v>
-      </c>
+      <c r="I25" s="12"/>
+      <c r="J25"/>
     </row>
     <row r="26" spans="1:10" ht="65.25" customHeight="1">
       <c r="A26" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" s="16"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F26" s="19"/>
-      <c r="G26" s="22">
-        <v>46203</v>
-      </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="11" t="s">
+      <c r="I26" s="12"/>
+      <c r="J26"/>
+    </row>
+    <row r="27" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="65.25" customHeight="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="11"/>
+      <c r="C27" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F27" s="16"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I27" s="12"/>
+      <c r="J27"/>
+    </row>
+    <row r="28" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A28" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="16"/>
+      <c r="H28" s="19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" s="16"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="16"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="16"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="65.25" customHeight="1">
+      <c r="A32" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="16"/>
+      <c r="H32" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="65.25" customHeight="1">
+      <c r="A33" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="16"/>
+      <c r="H33" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="65.25" customHeight="1">
+      <c r="A34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E34" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F34" s="16"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="65.25" customHeight="1">
+      <c r="A35" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="16"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="65.25" customHeight="1">
+      <c r="A36" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="16"/>
+      <c r="H36" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>